<commit_message>
fix: rehacer plantilla v1.1.1 sin romper protección ni validaciones
La v1.1.1 anterior quedó inutilizable: mi limpieza manual de las filas de
ejemplo borró celdas con estilos y estructura que la hoja protegida
necesitaba. Se rehace desde la v1.1.0 sana con UN solo cambio: la celda
J2 del CIF con formato texto (numFmtId 49). Protección, validaciones de
datos, tablas nombradas y fórmulas quedan intactas (3837 → 3838 celdas,
la diferencia es exactamente J2). Las filas de ejemplo se conservan: el
motor ya las ignora desde el fix del parser.
</commit_message>
<xml_diff>
--- a/docs/plantillas/CH-TPL-Depositos-v1.1.1.xlsx
+++ b/docs/plantillas/CH-TPL-Depositos-v1.1.1.xlsx
@@ -554,7 +554,7 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf applyNumberFormat="1" numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2773,10 +2773,27 @@
         <f>IF(7-(COUNTBLANK(J6:O6) + COUNTBLANK(Q6))&gt;0,1,"")</f>
         <v>1</v>
       </c>
+      <c r="J6" s="44">
+        <v>123456789</v>
+      </c>
+      <c r="K6" s="45">
+        <v>366789987</v>
+      </c>
+      <c r="L6" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="M6" s="46"/>
+      <c r="N6" s="46"/>
+      <c r="O6" s="46">
+        <v>200</v>
+      </c>
       <c r="P6" s="36">
         <f>SUM(M6:O6)</f>
         <v>200</v>
       </c>
+      <c r="Q6" s="45" t="s">
+        <v>13</v>
+      </c>
       <c r="R6" s="3"/>
       <c r="S6" s="14" t="s">
         <v>14</v>
@@ -2821,10 +2838,31 @@
         <f>IFERROR(IF(7-(COUNTBLANK(J7:O7) + COUNTBLANK(Q7))&gt;0,MAX($I$6:I6)+1,""),"")</f>
         <v>2</v>
       </c>
+      <c r="J7" s="44">
+        <v>123456789</v>
+      </c>
+      <c r="K7" s="45">
+        <v>366789987</v>
+      </c>
+      <c r="L7" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="M7" s="46"/>
+      <c r="N7" s="46">
+        <v>200</v>
+      </c>
+      <c r="O7" s="46">
+        <v>200</v>
+      </c>
       <c r="P7" s="36">
         <f t="shared" ref="P7:P70" si="5">SUM(M7:O7)</f>
         <v>400</v>
       </c>
+      <c r="Q7" s="45"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="16" t="s">
+        <v>12</v>
+      </c>
       <c r="T7" s="17">
         <f>SUM(T5:T6)</f>
         <v>1000</v>
@@ -2865,10 +2903,25 @@
         <f>IFERROR(IF(7-(COUNTBLANK(J8:O8) + COUNTBLANK(Q8))&gt;0,MAX($I$6:I7)+1,""),"")</f>
         <v>3</v>
       </c>
+      <c r="J8" s="44">
+        <v>123456789</v>
+      </c>
+      <c r="K8" s="45">
+        <v>366789988</v>
+      </c>
+      <c r="L8" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="M8" s="46"/>
+      <c r="N8" s="46"/>
+      <c r="O8" s="46">
+        <v>500</v>
+      </c>
       <c r="P8" s="36">
         <f t="shared" si="5"/>
         <v>500</v>
       </c>
+      <c r="Q8" s="45"/>
       <c r="R8" s="3"/>
       <c r="T8" s="2"/>
     </row>
@@ -2898,10 +2951,25 @@
         <f>IFERROR(IF(7-(COUNTBLANK(J9:O9) + COUNTBLANK(Q9))&gt;0,MAX($I$6:I8)+1,""),"")</f>
         <v>4</v>
       </c>
+      <c r="J9" s="44">
+        <v>123456789</v>
+      </c>
+      <c r="K9" s="45">
+        <v>366789988</v>
+      </c>
+      <c r="L9" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="M9" s="46"/>
+      <c r="N9" s="46"/>
+      <c r="O9" s="46">
+        <v>500</v>
+      </c>
       <c r="P9" s="36">
         <f t="shared" si="5"/>
         <v>500</v>
       </c>
+      <c r="Q9" s="45"/>
       <c r="R9" s="3"/>
       <c r="T9" s="2"/>
     </row>
@@ -11635,6 +11703,21 @@
       </c>
     </row>
     <row r="2" spans="1:8">
+      <c r="A2" s="47">
+        <v>2</v>
+      </c>
+      <c r="B2" s="48">
+        <v>120313</v>
+      </c>
+      <c r="C2" s="49" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="49" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="50">
+        <v>200</v>
+      </c>
       <c r="F2" s="8">
         <f>IF(AND(COUNTBLANK(A2:E2)&lt;&gt;5,COUNTBLANK(A2:E2)&lt;&gt;0),1,0)</f>
         <v>0</v>

</xml_diff>

<commit_message>
fix: celda J2 del CIF desbloqueada dentro de la hoja protegida
La hoja usa sheetProtection con celdas editables marcadas locked=0; la
J2 que agregué heredaba el bloqueo por defecto. El estilo nuevo combina
formato texto (numFmtId 49) con protection locked=0, igual que las
celdas que el cliente llena.
</commit_message>
<xml_diff>
--- a/docs/plantillas/CH-TPL-Depositos-v1.1.1.xlsx
+++ b/docs/plantillas/CH-TPL-Depositos-v1.1.1.xlsx
@@ -554,7 +554,9 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf applyNumberFormat="1" numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>

</xml_diff>